<commit_message>
Show daily customer recommendations with evidence
</commit_message>
<xml_diff>
--- a/dist/고객관리.xlsx
+++ b/dist/고객관리.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Rfcf84b752e024632"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R5a4d2cee53cf4ea7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -89,7 +89,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -121,10 +121,13 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -134,8 +137,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:J14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="10">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CustomerManagement" displayName="CustomerManagement" ref="A4:M14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
     <x:tableColumn id="1" name="발굴일"/>
     <x:tableColumn id="2" name="고객명"/>
     <x:tableColumn id="3" name="상권"/>
@@ -146,6 +149,9 @@
     <x:tableColumn id="8" name="다음 행동"/>
     <x:tableColumn id="9" name="마지막 연락일"/>
     <x:tableColumn id="10" name="발송 기록"/>
+    <x:tableColumn id="11" name="확인한 근거"/>
+    <x:tableColumn id="12" name="첫 상담에서 물어볼 내용"/>
+    <x:tableColumn id="13" name="근거 링크"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -350,18 +356,21 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="46" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="30" customHeight="1">
+    <x:row r="1">
       <x:c r="A1" s="4" t="str">
         <x:v>윤항무역 고객관리</x:v>
       </x:c>
@@ -374,10 +383,13 @@
       <x:c r="H1" s="4"/>
       <x:c r="I1" s="4"/>
       <x:c r="J1" s="4"/>
-    </x:row>
-    <x:row r="2" ht="32" customHeight="1">
+      <x:c r="K1" s="4"/>
+      <x:c r="L1" s="4"/>
+      <x:c r="M1" s="4"/>
+    </x:row>
+    <x:row r="2">
       <x:c r="A2" s="8" t="str">
-        <x:v>엑셀에서 후보를 관리한 뒤 웹앱의 ‘엑셀 가져오기’로 불러오세요. API 연동 전에는 매일 10명 후보를 이 표에 추가합니다.</x:v>
+        <x:v>하루 10명 후보를 검토하고 공개 근거·첫 상담 내용을 기록한 뒤 웹앱에서 엑셀 가져오기를 누르세요.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -388,8 +400,11 @@
       <x:c r="H2" s="8"/>
       <x:c r="I2" s="8"/>
       <x:c r="J2" s="8"/>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
+      <x:c r="K2" s="8"/>
+      <x:c r="L2" s="8"/>
+      <x:c r="M2" s="8"/>
+    </x:row>
+    <x:row r="4">
       <x:c r="A4" s="14" t="str">
         <x:v>발굴일</x:v>
       </x:c>
@@ -420,191 +435,278 @@
       <x:c r="J4" s="14" t="str">
         <x:v>발송 기록</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B5" s="16" t="str"/>
-      <x:c r="C5" s="16" t="str"/>
-      <x:c r="D5" s="16" t="str"/>
-      <x:c r="E5" s="16" t="str"/>
-      <x:c r="F5" s="16" t="str"/>
-      <x:c r="G5" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H5" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I5" s="17"/>
-      <x:c r="J5" s="16" t="str"/>
-    </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B6" s="16" t="str"/>
-      <x:c r="C6" s="16" t="str"/>
-      <x:c r="D6" s="16" t="str"/>
-      <x:c r="E6" s="16" t="str"/>
-      <x:c r="F6" s="16" t="str"/>
-      <x:c r="G6" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H6" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I6" s="17"/>
-      <x:c r="J6" s="16" t="str"/>
-    </x:row>
-    <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B7" s="16" t="str"/>
-      <x:c r="C7" s="16" t="str"/>
-      <x:c r="D7" s="16" t="str"/>
-      <x:c r="E7" s="16" t="str"/>
-      <x:c r="F7" s="16" t="str"/>
-      <x:c r="G7" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H7" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I7" s="17"/>
-      <x:c r="J7" s="16" t="str"/>
-    </x:row>
-    <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B8" s="16" t="str"/>
-      <x:c r="C8" s="16" t="str"/>
-      <x:c r="D8" s="16" t="str"/>
-      <x:c r="E8" s="16" t="str"/>
-      <x:c r="F8" s="16" t="str"/>
-      <x:c r="G8" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H8" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I8" s="17"/>
-      <x:c r="J8" s="16" t="str"/>
-    </x:row>
-    <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B9" s="16" t="str"/>
-      <x:c r="C9" s="16" t="str"/>
-      <x:c r="D9" s="16" t="str"/>
-      <x:c r="E9" s="16" t="str"/>
-      <x:c r="F9" s="16" t="str"/>
-      <x:c r="G9" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H9" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I9" s="17"/>
-      <x:c r="J9" s="16" t="str"/>
-    </x:row>
-    <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B10" s="16" t="str"/>
-      <x:c r="C10" s="16" t="str"/>
-      <x:c r="D10" s="16" t="str"/>
-      <x:c r="E10" s="16" t="str"/>
-      <x:c r="F10" s="16" t="str"/>
-      <x:c r="G10" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H10" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I10" s="17"/>
-      <x:c r="J10" s="16" t="str"/>
-    </x:row>
-    <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B11" s="16" t="str"/>
-      <x:c r="C11" s="16" t="str"/>
-      <x:c r="D11" s="16" t="str"/>
-      <x:c r="E11" s="16" t="str"/>
-      <x:c r="F11" s="16" t="str"/>
-      <x:c r="G11" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H11" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I11" s="17"/>
-      <x:c r="J11" s="16" t="str"/>
-    </x:row>
-    <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B12" s="16" t="str"/>
-      <x:c r="C12" s="16" t="str"/>
-      <x:c r="D12" s="16" t="str"/>
-      <x:c r="E12" s="16" t="str"/>
-      <x:c r="F12" s="16" t="str"/>
-      <x:c r="G12" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H12" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I12" s="17"/>
-      <x:c r="J12" s="16" t="str"/>
-    </x:row>
-    <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B13" s="16" t="str"/>
-      <x:c r="C13" s="16" t="str"/>
-      <x:c r="D13" s="16" t="str"/>
-      <x:c r="E13" s="16" t="str"/>
-      <x:c r="F13" s="16" t="str"/>
-      <x:c r="G13" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H13" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I13" s="17"/>
-      <x:c r="J13" s="16" t="str"/>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="17" t="d">
-        <x:v>2026-10-11T12:31:57.052Z</x:v>
-      </x:c>
-      <x:c r="B14" s="16" t="str"/>
-      <x:c r="C14" s="16" t="str"/>
-      <x:c r="D14" s="16" t="str"/>
-      <x:c r="E14" s="16" t="str"/>
-      <x:c r="F14" s="16" t="str"/>
-      <x:c r="G14" s="16" t="str">
-        <x:v>검토 필요</x:v>
-      </x:c>
-      <x:c r="H14" s="16" t="str">
-        <x:v>연락처 확인</x:v>
-      </x:c>
-      <x:c r="I14" s="17"/>
-      <x:c r="J14" s="16" t="str"/>
+      <x:c r="K4" s="14" t="str">
+        <x:v>확인한 근거</x:v>
+      </x:c>
+      <x:c r="L4" s="14" t="str">
+        <x:v>첫 상담에서 물어볼 내용</x:v>
+      </x:c>
+      <x:c r="M4" s="14" t="str">
+        <x:v>근거 링크</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B5" s="17" t="str">
+        <x:v>뉴골드</x:v>
+      </x:c>
+      <x:c r="C5" s="17" t="str">
+        <x:v>통일상가</x:v>
+      </x:c>
+      <x:c r="D5" s="17" t="str">
+        <x:v>남성 캐주얼 바지</x:v>
+      </x:c>
+      <x:c r="E5" s="17" t="str"/>
+      <x:c r="F5" s="17" t="str"/>
+      <x:c r="G5" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H5" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I5" s="18"/>
+      <x:c r="J5" s="17" t="str"/>
+      <x:c r="K5" s="17" t="str">
+        <x:v>2025년 11월 매장 채용 공고에서 남성 캐주얼 바지 도매업체라고 소개</x:v>
+      </x:c>
+      <x:c r="L5" s="17" t="str">
+        <x:v>가을·겨울 바지의 중국 생산 여부와 주력 상품 발주량</x:v>
+      </x:c>
+      <x:c r="M5" s="17" t="str">
+        <x:v>공개 채용 공고 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B6" s="17" t="str">
+        <x:v>마스터베어</x:v>
+      </x:c>
+      <x:c r="C6" s="17" t="str">
+        <x:v>통일상가 B동 2층 2100호</x:v>
+      </x:c>
+      <x:c r="D6" s="17" t="str">
+        <x:v>남녀 F/W</x:v>
+      </x:c>
+      <x:c r="E6" s="17" t="str"/>
+      <x:c r="F6" s="17" t="str"/>
+      <x:c r="G6" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H6" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I6" s="18"/>
+      <x:c r="J6" s="17" t="str"/>
+      <x:c r="K6" s="17" t="str">
+        <x:v>공식 사이트에 매장 주소와 남녀 가을·겨울 상품 구분 공개</x:v>
+      </x:c>
+      <x:c r="L6" s="17" t="str">
+        <x:v>바지·재킷 중 외부 생산 협력을 검토할 품목이 있는지</x:v>
+      </x:c>
+      <x:c r="M6" s="17" t="str">
+        <x:v>공식 사이트 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B7" s="17" t="str">
+        <x:v>ELTOO(엘트)</x:v>
+      </x:c>
+      <x:c r="C7" s="17" t="str">
+        <x:v>누존 1층</x:v>
+      </x:c>
+      <x:c r="D7" s="17" t="str">
+        <x:v>여성 바지</x:v>
+      </x:c>
+      <x:c r="E7" s="17" t="str"/>
+      <x:c r="F7" s="17" t="str"/>
+      <x:c r="G7" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H7" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I7" s="18"/>
+      <x:c r="J7" s="17" t="str"/>
+      <x:c r="K7" s="17" t="str">
+        <x:v>2025년 1월 매장 채용 공고에서 여성 바지 전문 매장이라고 소개</x:v>
+      </x:c>
+      <x:c r="L7" s="17" t="str">
+        <x:v>여성 팬츠 생산 방식과 시즌별 예상 물량</x:v>
+      </x:c>
+      <x:c r="M7" s="17" t="str">
+        <x:v>공개 채용 공고 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B8" s="17" t="str">
+        <x:v>하프인치</x:v>
+      </x:c>
+      <x:c r="C8" s="17" t="str">
+        <x:v>디오트</x:v>
+      </x:c>
+      <x:c r="D8" s="17" t="str">
+        <x:v>바지</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="str"/>
+      <x:c r="F8" s="17" t="str"/>
+      <x:c r="G8" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H8" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I8" s="18"/>
+      <x:c r="J8" s="17" t="str"/>
+      <x:c r="K8" s="17" t="str">
+        <x:v>2026년 1월 공고에서 바지 전문 매장과 원단·패턴·메인공장 운영 관계를 설명</x:v>
+      </x:c>
+      <x:c r="L8" s="17" t="str">
+        <x:v>기존 공장 외 추가 생산이나 별도 품목 수요가 있는지</x:v>
+      </x:c>
+      <x:c r="M8" s="17" t="str">
+        <x:v>공개 채용 공고 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str"/>
+      <x:c r="C9" s="17" t="str"/>
+      <x:c r="D9" s="17" t="str"/>
+      <x:c r="E9" s="17" t="str"/>
+      <x:c r="F9" s="17" t="str"/>
+      <x:c r="G9" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H9" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I9" s="18"/>
+      <x:c r="J9" s="17" t="str"/>
+      <x:c r="K9" s="17" t="str"/>
+      <x:c r="L9" s="17" t="str"/>
+      <x:c r="M9" s="17" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str"/>
+      <x:c r="C10" s="17" t="str"/>
+      <x:c r="D10" s="17" t="str"/>
+      <x:c r="E10" s="17" t="str"/>
+      <x:c r="F10" s="17" t="str"/>
+      <x:c r="G10" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H10" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I10" s="18"/>
+      <x:c r="J10" s="17" t="str"/>
+      <x:c r="K10" s="17" t="str"/>
+      <x:c r="L10" s="17" t="str"/>
+      <x:c r="M10" s="17" t="str"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str"/>
+      <x:c r="C11" s="17" t="str"/>
+      <x:c r="D11" s="17" t="str"/>
+      <x:c r="E11" s="17" t="str"/>
+      <x:c r="F11" s="17" t="str"/>
+      <x:c r="G11" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H11" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I11" s="18"/>
+      <x:c r="J11" s="17" t="str"/>
+      <x:c r="K11" s="17" t="str"/>
+      <x:c r="L11" s="17" t="str"/>
+      <x:c r="M11" s="17" t="str"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="str"/>
+      <x:c r="C12" s="17" t="str"/>
+      <x:c r="D12" s="17" t="str"/>
+      <x:c r="E12" s="17" t="str"/>
+      <x:c r="F12" s="17" t="str"/>
+      <x:c r="G12" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H12" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I12" s="18"/>
+      <x:c r="J12" s="17" t="str"/>
+      <x:c r="K12" s="17" t="str"/>
+      <x:c r="L12" s="17" t="str"/>
+      <x:c r="M12" s="17" t="str"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="str"/>
+      <x:c r="C13" s="17" t="str"/>
+      <x:c r="D13" s="17" t="str"/>
+      <x:c r="E13" s="17" t="str"/>
+      <x:c r="F13" s="17" t="str"/>
+      <x:c r="G13" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H13" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I13" s="18"/>
+      <x:c r="J13" s="17" t="str"/>
+      <x:c r="K13" s="17" t="str"/>
+      <x:c r="L13" s="17" t="str"/>
+      <x:c r="M13" s="17" t="str"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="18" t="d">
+        <x:v>2026-10-11T12:40:53.671Z</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str"/>
+      <x:c r="C14" s="17" t="str"/>
+      <x:c r="D14" s="17" t="str"/>
+      <x:c r="E14" s="17" t="str"/>
+      <x:c r="F14" s="17" t="str"/>
+      <x:c r="G14" s="17" t="str">
+        <x:v>검토 필요</x:v>
+      </x:c>
+      <x:c r="H14" s="17" t="str">
+        <x:v>연락처 확인</x:v>
+      </x:c>
+      <x:c r="I14" s="18"/>
+      <x:c r="J14" s="17" t="str"/>
+      <x:c r="K14" s="17" t="str"/>
+      <x:c r="L14" s="17" t="str"/>
+      <x:c r="M14" s="17" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:J1"/>
-    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A1:M1"/>
+    <x:mergeCell ref="A2:M2"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="G5:G1000">
@@ -613,7 +715,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R05ebfbc5016f4ab9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb823f3d7590d4cbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Populate ten daily customer recommendations
</commit_message>
<xml_diff>
--- a/dist/고객관리.xlsx
+++ b/dist/고객관리.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="R5a4d2cee53cf4ea7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객관리" sheetId="1" r:id="Ra410995f2eb14846"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -356,18 +356,18 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="17" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="46" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="48" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="42" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="62" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -389,7 +389,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="8" t="str">
-        <x:v>하루 10명 후보를 검토하고 공개 근거·첫 상담 내용을 기록한 뒤 웹앱에서 엑셀 가져오기를 누르세요.</x:v>
+        <x:v>오늘 추천 고객 10명입니다. 공개 근거를 확인하고 개별 매장명·담당자·연락처를 확인한 뒤 웹앱으로 가져오세요.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -447,7 +447,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
       </x:c>
       <x:c r="B5" s="17" t="str">
         <x:v>뉴골드</x:v>
@@ -475,12 +475,12 @@
         <x:v>가을·겨울 바지의 중국 생산 여부와 주력 상품 발주량</x:v>
       </x:c>
       <x:c r="M5" s="17" t="str">
-        <x:v>공개 채용 공고 확인</x:v>
+        <x:v>사용자 제공 공개 공고 내용</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
       </x:c>
       <x:c r="B6" s="17" t="str">
         <x:v>마스터베어</x:v>
@@ -508,12 +508,12 @@
         <x:v>바지·재킷 중 외부 생산 협력을 검토할 품목이 있는지</x:v>
       </x:c>
       <x:c r="M6" s="17" t="str">
-        <x:v>공식 사이트 확인</x:v>
+        <x:v>사용자 제공 공개 사이트 내용</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
       </x:c>
       <x:c r="B7" s="17" t="str">
         <x:v>ELTOO(엘트)</x:v>
@@ -541,12 +541,12 @@
         <x:v>여성 팬츠 생산 방식과 시즌별 예상 물량</x:v>
       </x:c>
       <x:c r="M7" s="17" t="str">
-        <x:v>공개 채용 공고 확인</x:v>
+        <x:v>사용자 제공 공개 공고 내용</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
       </x:c>
       <x:c r="B8" s="17" t="str">
         <x:v>하프인치</x:v>
@@ -574,16 +574,22 @@
         <x:v>기존 공장 외 추가 생산이나 별도 품목 수요가 있는지</x:v>
       </x:c>
       <x:c r="M8" s="17" t="str">
-        <x:v>공개 채용 공고 확인</x:v>
+        <x:v>사용자 제공 공개 공고 내용</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
-      </x:c>
-      <x:c r="B9" s="17" t="str"/>
-      <x:c r="C9" s="17" t="str"/>
-      <x:c r="D9" s="17" t="str"/>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
+      </x:c>
+      <x:c r="B9" s="17" t="str">
+        <x:v>더베스트오버초이스</x:v>
+      </x:c>
+      <x:c r="C9" s="17" t="str">
+        <x:v>통일상가 B동 2층 250·251</x:v>
+      </x:c>
+      <x:c r="D9" s="17" t="str">
+        <x:v>가을·겨울 바지</x:v>
+      </x:c>
       <x:c r="E9" s="17" t="str"/>
       <x:c r="F9" s="17" t="str"/>
       <x:c r="G9" s="17" t="str">
@@ -594,114 +600,180 @@
       </x:c>
       <x:c r="I9" s="18"/>
       <x:c r="J9" s="17" t="str"/>
-      <x:c r="K9" s="17" t="str"/>
-      <x:c r="L9" s="17" t="str"/>
-      <x:c r="M9" s="17" t="str"/>
+      <x:c r="K9" s="17" t="str">
+        <x:v>기존 고객관리 목록에 등록된 매장 후보</x:v>
+      </x:c>
+      <x:c r="L9" s="17" t="str">
+        <x:v>가을·겨울 바지 샘플 확인 후 생산 상담 가능 여부</x:v>
+      </x:c>
+      <x:c r="M9" s="17" t="str">
+        <x:v>내 고객관리 기록</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
-      </x:c>
-      <x:c r="B10" s="17" t="str"/>
-      <x:c r="C10" s="17" t="str"/>
-      <x:c r="D10" s="17" t="str"/>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
+      </x:c>
+      <x:c r="B10" s="17" t="str">
+        <x:v>디오트 여성 팬츠 매장 후보</x:v>
+      </x:c>
+      <x:c r="C10" s="17" t="str">
+        <x:v>디오트</x:v>
+      </x:c>
+      <x:c r="D10" s="17" t="str">
+        <x:v>여성복·바지</x:v>
+      </x:c>
       <x:c r="E10" s="17" t="str"/>
       <x:c r="F10" s="17" t="str"/>
       <x:c r="G10" s="17" t="str">
         <x:v>검토 필요</x:v>
       </x:c>
       <x:c r="H10" s="17" t="str">
-        <x:v>연락처 확인</x:v>
+        <x:v>개별 매장명 확인</x:v>
       </x:c>
       <x:c r="I10" s="18"/>
       <x:c r="J10" s="17" t="str"/>
-      <x:c r="K10" s="17" t="str"/>
-      <x:c r="L10" s="17" t="str"/>
-      <x:c r="M10" s="17" t="str"/>
+      <x:c r="K10" s="17" t="str">
+        <x:v>디오트가 동대문 주요 도매시장으로 소개되는 시장 단위 후보</x:v>
+      </x:c>
+      <x:c r="L10" s="17" t="str">
+        <x:v>개별 매장명과 담당자, 여성 팬츠 외부 생산 협력 여부를 확인</x:v>
+      </x:c>
+      <x:c r="M10" s="17" t="str">
+        <x:v>https://b-flow.co.kr/posts/39</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
-      </x:c>
-      <x:c r="B11" s="17" t="str"/>
-      <x:c r="C11" s="17" t="str"/>
-      <x:c r="D11" s="17" t="str"/>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
+      </x:c>
+      <x:c r="B11" s="17" t="str">
+        <x:v>누죤 여성 캐주얼 매장 후보</x:v>
+      </x:c>
+      <x:c r="C11" s="17" t="str">
+        <x:v>누죤</x:v>
+      </x:c>
+      <x:c r="D11" s="17" t="str">
+        <x:v>여성 캐주얼·바지</x:v>
+      </x:c>
       <x:c r="E11" s="17" t="str"/>
       <x:c r="F11" s="17" t="str"/>
       <x:c r="G11" s="17" t="str">
         <x:v>검토 필요</x:v>
       </x:c>
       <x:c r="H11" s="17" t="str">
-        <x:v>연락처 확인</x:v>
+        <x:v>개별 매장명 확인</x:v>
       </x:c>
       <x:c r="I11" s="18"/>
       <x:c r="J11" s="17" t="str"/>
-      <x:c r="K11" s="17" t="str"/>
-      <x:c r="L11" s="17" t="str"/>
-      <x:c r="M11" s="17" t="str"/>
+      <x:c r="K11" s="17" t="str">
+        <x:v>누죤이 동대문 의류 도매 상권으로 소개되는 시장 단위 후보</x:v>
+      </x:c>
+      <x:c r="L11" s="17" t="str">
+        <x:v>주력 품목과 가을·겨울 바지 생산 수요를 확인</x:v>
+      </x:c>
+      <x:c r="M11" s="17" t="str">
+        <x:v>https://www.i-boss.co.kr/ab-1486517-2773</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
-      </x:c>
-      <x:c r="B12" s="17" t="str"/>
-      <x:c r="C12" s="17" t="str"/>
-      <x:c r="D12" s="17" t="str"/>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
+      </x:c>
+      <x:c r="B12" s="17" t="str">
+        <x:v>청평화상가 바지 매장 후보</x:v>
+      </x:c>
+      <x:c r="C12" s="17" t="str">
+        <x:v>청평화상가</x:v>
+      </x:c>
+      <x:c r="D12" s="17" t="str">
+        <x:v>바지·재킷</x:v>
+      </x:c>
       <x:c r="E12" s="17" t="str"/>
       <x:c r="F12" s="17" t="str"/>
       <x:c r="G12" s="17" t="str">
         <x:v>검토 필요</x:v>
       </x:c>
       <x:c r="H12" s="17" t="str">
-        <x:v>연락처 확인</x:v>
+        <x:v>개별 매장명 확인</x:v>
       </x:c>
       <x:c r="I12" s="18"/>
       <x:c r="J12" s="17" t="str"/>
-      <x:c r="K12" s="17" t="str"/>
-      <x:c r="L12" s="17" t="str"/>
-      <x:c r="M12" s="17" t="str"/>
+      <x:c r="K12" s="17" t="str">
+        <x:v>청평화상가가 동대문 주요 도매 상권으로 안내되는 시장 단위 후보</x:v>
+      </x:c>
+      <x:c r="L12" s="17" t="str">
+        <x:v>바지·재킷 중 추가 생산이 필요한 품목을 확인</x:v>
+      </x:c>
+      <x:c r="M12" s="17" t="str">
+        <x:v>https://my-luggage-app.duckdns.org/blog/dongdaemun-dawn-shopping-guide-2026</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
-      </x:c>
-      <x:c r="B13" s="17" t="str"/>
-      <x:c r="C13" s="17" t="str"/>
-      <x:c r="D13" s="17" t="str"/>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
+      </x:c>
+      <x:c r="B13" s="17" t="str">
+        <x:v>신평화시장 캐주얼 매장 후보</x:v>
+      </x:c>
+      <x:c r="C13" s="17" t="str">
+        <x:v>신평화시장</x:v>
+      </x:c>
+      <x:c r="D13" s="17" t="str">
+        <x:v>캐주얼·F/W</x:v>
+      </x:c>
       <x:c r="E13" s="17" t="str"/>
       <x:c r="F13" s="17" t="str"/>
       <x:c r="G13" s="17" t="str">
         <x:v>검토 필요</x:v>
       </x:c>
       <x:c r="H13" s="17" t="str">
-        <x:v>연락처 확인</x:v>
+        <x:v>개별 매장명 확인</x:v>
       </x:c>
       <x:c r="I13" s="18"/>
       <x:c r="J13" s="17" t="str"/>
-      <x:c r="K13" s="17" t="str"/>
-      <x:c r="L13" s="17" t="str"/>
-      <x:c r="M13" s="17" t="str"/>
+      <x:c r="K13" s="17" t="str">
+        <x:v>신평화시장이 동대문 의류 도매 상권으로 안내되는 시장 단위 후보</x:v>
+      </x:c>
+      <x:c r="L13" s="17" t="str">
+        <x:v>거래 방식과 시즌별 발주 일정을 확인</x:v>
+      </x:c>
+      <x:c r="M13" s="17" t="str">
+        <x:v>https://my-luggage-app.duckdns.org/blog/dongdaemun-dawn-shopping-guide-2026</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="18" t="d">
-        <x:v>2026-10-11T12:40:53.671Z</x:v>
-      </x:c>
-      <x:c r="B14" s="17" t="str"/>
-      <x:c r="C14" s="17" t="str"/>
-      <x:c r="D14" s="17" t="str"/>
+        <x:v>2026-10-11T12:43:17.021Z</x:v>
+      </x:c>
+      <x:c r="B14" s="17" t="str">
+        <x:v>유어스(U:US) F/W 매장 후보</x:v>
+      </x:c>
+      <x:c r="C14" s="17" t="str">
+        <x:v>유어스(U:US)</x:v>
+      </x:c>
+      <x:c r="D14" s="17" t="str">
+        <x:v>여성·남성 F/W</x:v>
+      </x:c>
       <x:c r="E14" s="17" t="str"/>
       <x:c r="F14" s="17" t="str"/>
       <x:c r="G14" s="17" t="str">
         <x:v>검토 필요</x:v>
       </x:c>
       <x:c r="H14" s="17" t="str">
-        <x:v>연락처 확인</x:v>
+        <x:v>개별 매장명 확인</x:v>
       </x:c>
       <x:c r="I14" s="18"/>
       <x:c r="J14" s="17" t="str"/>
-      <x:c r="K14" s="17" t="str"/>
-      <x:c r="L14" s="17" t="str"/>
-      <x:c r="M14" s="17" t="str"/>
+      <x:c r="K14" s="17" t="str">
+        <x:v>유어스가 동대문 대표 도매 상권으로 소개되는 시장 단위 후보</x:v>
+      </x:c>
+      <x:c r="L14" s="17" t="str">
+        <x:v>개별 매장명과 외부 생산·샘플 상담 가능 여부를 확인</x:v>
+      </x:c>
+      <x:c r="M14" s="17" t="str">
+        <x:v>https://my-luggage-app.duckdns.org/blog/dongdaemun-dawn-shopping-guide-2026</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -715,7 +787,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb823f3d7590d4cbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5dacd06d25164a11"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>